<commit_message>
added features and streamlit app
</commit_message>
<xml_diff>
--- a/output/Job_Applications_Tracker_2026-03.xlsx
+++ b/output/Job_Applications_Tracker_2026-03.xlsx
@@ -34,7 +34,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,11 +44,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -69,13 +64,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -458,7 +452,7 @@
     <col width="40" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
     <col width="40" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="21" customWidth="1" min="17" max="17"/>
@@ -610,12 +604,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Applied</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>DEMO-20260328-5578</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -689,12 +683,12 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Applied</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>DEMO-20260328-6391</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -710,454 +704,454 @@
       <c r="Q3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>03/28/2026</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>IC Design Engineering Intern</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>NVIDIA</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Technology / Semiconductor</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Santa Clara, CA</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>https://nvidia.com/careers/intern-ic</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>https://www.nvidia.com</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="J4" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>Score 73 below threshold or max_apps reached</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Score 73 below threshold or max applications reached</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>04/04/2026</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>03/28/2026</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Mixed-Signal IC Design Intern</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Apple</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Technology / Semiconductor</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Cupertino, CA</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>https://apple.com/jobs</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>https://www.apple.com</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="J5" s="3" t="n">
+      <c r="J5" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="K5" s="3" t="inlineStr"/>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>Score 73 below threshold or max_apps reached</t>
-        </is>
-      </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>Score 73 below threshold or max applications reached</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>04/04/2026</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>03/28/2026</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>EE Hardware Design Intern</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Samsung Semiconductors</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Technology / Semiconductor</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>San Jose, CA</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>https://samsung.com/us/careers</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>https://www.samsungsemiconductors.com</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="J6" s="3" t="n">
+      <c r="J6" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="K6" s="3" t="inlineStr"/>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
-        <is>
-          <t>Score 73 below threshold or max_apps reached</t>
-        </is>
-      </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>Score 73 below threshold or max applications reached</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>04/04/2026</t>
         </is>
       </c>
-      <c r="Q6" s="3" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>03/28/2026</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Semiconductor Process Engineering Intern</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Micron Technology</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Technology / Semiconductor</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Boise, ID</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>https://micron.com/careers</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>https://www.microntechnology.com</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Glassdoor</t>
         </is>
       </c>
-      <c r="J7" s="3" t="n">
+      <c r="J7" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="K7" s="3" t="inlineStr"/>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
-        <is>
-          <t>Score 68 below threshold or max_apps reached</t>
-        </is>
-      </c>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Score 68 below threshold or max applications reached</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>04/04/2026</t>
         </is>
       </c>
-      <c r="Q7" s="3" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>03/28/2026</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Photonics Engineering Intern</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Lumentum</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Technology / Semiconductor</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>San Jose, CA</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>https://lumentum.com/careers</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>https://www.lumentum.com</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Indeed</t>
         </is>
       </c>
-      <c r="J8" s="3" t="n">
+      <c r="J8" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="K8" s="3" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O8" s="3" t="inlineStr">
-        <is>
-          <t>Score 63 below threshold or max_apps reached</t>
-        </is>
-      </c>
-      <c r="P8" s="3" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Score 63 below threshold or max applications reached</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>04/04/2026</t>
         </is>
       </c>
-      <c r="Q8" s="3" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>03/28/2026</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Nanoelectronics Research Intern</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>IBM Research</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Technology / Semiconductor</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Yorktown Heights, NY</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>https://research.ibm.com/careers</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>https://www.ibmresearch.com</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Handshake</t>
         </is>
       </c>
-      <c r="J9" s="3" t="n">
+      <c r="J9" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="K9" s="3" t="inlineStr"/>
-      <c r="L9" s="3" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
       </c>
-      <c r="N9" s="3" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O9" s="3" t="inlineStr">
-        <is>
-          <t>Score 63 below threshold or max_apps reached</t>
-        </is>
-      </c>
-      <c r="P9" s="3" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Score 63 below threshold or max applications reached</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t>04/04/2026</t>
         </is>
       </c>
-      <c r="Q9" s="3" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1174,12 +1168,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -1214,7 +1208,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1234,7 +1228,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
bug fixes to streamlit
</commit_message>
<xml_diff>
--- a/output/Job_Applications_Tracker_2026-03.xlsx
+++ b/output/Job_Applications_Tracker_2026-03.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -556,12 +556,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>FPGA/Hardware Engineering Intern</t>
+          <t>Mixed-Signal IC Design Intern</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -571,30 +571,30 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Hillsboro, OR</t>
+          <t>Cupertino, CA</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>https://intel.com/jobs</t>
+          <t>https://apple.com/jobs</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://www.intel.com</t>
+          <t>https://www.apple.com</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Handshake</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Your_Name_Resume_Intel_FPGA_Hardware_Engineering_Intern.txt</t>
+          <t>Your_Name_Resume_Apple_Mixed-Signal_IC_Design_Intern.txt</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>ATS gaps: Linux</t>
+          <t>ATS gaps: ARM Microcontrollers, FPGA SystemVerilog</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Hardware Engineering Intern</t>
+          <t>Semiconductor Process Engineering Intern</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Micron Technology</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -650,30 +650,30 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Redmond, WA</t>
+          <t>Boise, ID</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>https://microsoft.com/careers</t>
+          <t>https://micron.com/careers</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://www.microsoft.com</t>
+          <t>https://www.microntechnology.com</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Your_Name_Resume_Microsoft_Hardware_Engineering_Intern.txt</t>
+          <t>Your_Name_Resume_Micron_Technology_Semiconductor_Process_Engineering_Intern.txt</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>ATS gaps: C++, Schematic</t>
+          <t>ATS gaps: FPGA SystemVerilog</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>IC Design Engineering Intern</t>
+          <t>EE Hardware Design Intern</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Samsung Semiconductors</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -729,17 +729,17 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Santa Clara, CA</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>https://nvidia.com/careers/intern-ic</t>
+          <t>https://samsung.com/us/careers</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://www.nvidia.com</t>
+          <t>https://www.samsungsemiconductors.com</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -748,9 +748,13 @@
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>73</v>
-      </c>
-      <c r="K4" s="2" t="inlineStr"/>
+        <v>75</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Your_Name_Resume_Samsung_Semiconductors_EE_Hardware_Design_Intern.txt</t>
+        </is>
+      </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -768,7 +772,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Score 73 below threshold or max applications reached</t>
+          <t>ATS gaps: SPICE, MATLAB</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -789,12 +793,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Mixed-Signal IC Design Intern</t>
+          <t>IC Design Engineering Intern</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -804,17 +808,17 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Cupertino, CA</t>
+          <t>Santa Clara, CA</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>https://apple.com/jobs</t>
+          <t>https://nvidia.com/careers/intern-ic</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>https://www.apple.com</t>
+          <t>https://www.nvidia.com</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -823,7 +827,7 @@
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
@@ -843,7 +847,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Score 73 below threshold or max applications reached</t>
+          <t>Score 72 below threshold or max applications reached</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -864,12 +868,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>EE Hardware Design Intern</t>
+          <t>Photonics Engineering Intern</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Samsung Semiconductors</t>
+          <t>Lumentum</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -884,21 +888,21 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>https://samsung.com/us/careers</t>
+          <t>https://lumentum.com/careers</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://www.samsungsemiconductors.com</t>
+          <t>https://www.lumentum.com</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
@@ -918,7 +922,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Score 73 below threshold or max applications reached</t>
+          <t>Score 68 below threshold or max applications reached</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -939,12 +943,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Semiconductor Process Engineering Intern</t>
+          <t>Nanoelectronics Research Intern</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Micron Technology</t>
+          <t>IBM Research</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -954,26 +958,26 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Boise, ID</t>
+          <t>Yorktown Heights, NY</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://micron.com/careers</t>
+          <t>https://research.ibm.com/careers</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://www.microntechnology.com</t>
+          <t>https://www.ibmresearch.com</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Handshake</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
@@ -993,7 +997,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Score 68 below threshold or max applications reached</t>
+          <t>Score 63 below threshold or max applications reached</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1014,12 +1018,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Photonics Engineering Intern</t>
+          <t>Hardware Engineering Intern</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Lumentum</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1029,17 +1033,17 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>Redmond, WA</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://lumentum.com/careers</t>
+          <t>https://microsoft.com/careers</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://www.lumentum.com</t>
+          <t>https://www.microsoft.com</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1048,7 +1052,7 @@
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
@@ -1068,7 +1072,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Score 63 below threshold or max applications reached</t>
+          <t>Score 60 below threshold or max applications reached</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1077,81 +1081,6 @@
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>03/28/2026</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Nanoelectronics Research Intern</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>IBM Research</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Technology / Semiconductor</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Yorktown Heights, NY</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>https://research.ibm.com/careers</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.ibmresearch.com</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Handshake</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Skipped</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>Score 63 below threshold or max applications reached</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>04/04/2026</t>
-        </is>
-      </c>
-      <c r="Q9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1198,7 +1127,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -1228,7 +1157,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -1239,7 +1168,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>71.8</t>
+          <t>72.3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "bug fixes to streamlit"
This reverts commit a76b8dee8571f29cc5f5f6ed0fb612e4e50323aa.

A
Revert
</commit_message>
<xml_diff>
--- a/output/Job_Applications_Tracker_2026-03.xlsx
+++ b/output/Job_Applications_Tracker_2026-03.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -556,12 +556,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Mixed-Signal IC Design Intern</t>
+          <t>FPGA/Hardware Engineering Intern</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -571,30 +571,30 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Cupertino, CA</t>
+          <t>Hillsboro, OR</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>https://apple.com/jobs</t>
+          <t>https://intel.com/jobs</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://www.apple.com</t>
+          <t>https://www.intel.com</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Handshake</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Your_Name_Resume_Apple_Mixed-Signal_IC_Design_Intern.txt</t>
+          <t>Your_Name_Resume_Intel_FPGA_Hardware_Engineering_Intern.txt</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>ATS gaps: ARM Microcontrollers, FPGA SystemVerilog</t>
+          <t>ATS gaps: Linux</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Semiconductor Process Engineering Intern</t>
+          <t>Hardware Engineering Intern</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Micron Technology</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -650,30 +650,30 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Boise, ID</t>
+          <t>Redmond, WA</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>https://micron.com/careers</t>
+          <t>https://microsoft.com/careers</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://www.microntechnology.com</t>
+          <t>https://www.microsoft.com</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Indeed</t>
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Your_Name_Resume_Micron_Technology_Semiconductor_Process_Engineering_Intern.txt</t>
+          <t>Your_Name_Resume_Microsoft_Hardware_Engineering_Intern.txt</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>ATS gaps: FPGA SystemVerilog</t>
+          <t>ATS gaps: C++, Schematic</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -714,12 +714,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>EE Hardware Design Intern</t>
+          <t>IC Design Engineering Intern</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Samsung Semiconductors</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -729,17 +729,17 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>San Jose, CA</t>
+          <t>Santa Clara, CA</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>https://samsung.com/us/careers</t>
+          <t>https://nvidia.com/careers/intern-ic</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://www.samsungsemiconductors.com</t>
+          <t>https://www.nvidia.com</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -748,13 +748,9 @@
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Your_Name_Resume_Samsung_Semiconductors_EE_Hardware_Design_Intern.txt</t>
-        </is>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -772,7 +768,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>ATS gaps: SPICE, MATLAB</t>
+          <t>Score 73 below threshold or max applications reached</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -793,12 +789,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>IC Design Engineering Intern</t>
+          <t>Mixed-Signal IC Design Intern</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -808,17 +804,17 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Santa Clara, CA</t>
+          <t>Cupertino, CA</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>https://nvidia.com/careers/intern-ic</t>
+          <t>https://apple.com/jobs</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>https://www.nvidia.com</t>
+          <t>https://www.apple.com</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -827,7 +823,7 @@
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
@@ -847,7 +843,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Score 72 below threshold or max applications reached</t>
+          <t>Score 73 below threshold or max applications reached</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -868,12 +864,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Photonics Engineering Intern</t>
+          <t>EE Hardware Design Intern</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Lumentum</t>
+          <t>Samsung Semiconductors</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -888,21 +884,21 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>https://lumentum.com/careers</t>
+          <t>https://samsung.com/us/careers</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://www.lumentum.com</t>
+          <t>https://www.samsungsemiconductors.com</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
@@ -922,7 +918,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Score 68 below threshold or max applications reached</t>
+          <t>Score 73 below threshold or max applications reached</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -943,12 +939,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Nanoelectronics Research Intern</t>
+          <t>Semiconductor Process Engineering Intern</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>IBM Research</t>
+          <t>Micron Technology</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -958,26 +954,26 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Yorktown Heights, NY</t>
+          <t>Boise, ID</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://research.ibm.com/careers</t>
+          <t>https://micron.com/careers</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://www.ibmresearch.com</t>
+          <t>https://www.microntechnology.com</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Handshake</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
@@ -997,7 +993,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Score 63 below threshold or max applications reached</t>
+          <t>Score 68 below threshold or max applications reached</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1018,12 +1014,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Hardware Engineering Intern</t>
+          <t>Photonics Engineering Intern</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Lumentum</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1033,17 +1029,17 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Redmond, WA</t>
+          <t>San Jose, CA</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://microsoft.com/careers</t>
+          <t>https://lumentum.com/careers</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://www.microsoft.com</t>
+          <t>https://www.lumentum.com</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1052,7 +1048,7 @@
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
@@ -1072,7 +1068,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Score 60 below threshold or max applications reached</t>
+          <t>Score 63 below threshold or max applications reached</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1081,6 +1077,81 @@
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>03/28/2026</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Nanoelectronics Research Intern</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>IBM Research</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Technology / Semiconductor</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Yorktown Heights, NY</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>https://research.ibm.com/careers</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ibmresearch.com</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Handshake</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Score 63 below threshold or max applications reached</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1127,7 +1198,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -1157,7 +1228,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -1168,7 +1239,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>71.8</t>
         </is>
       </c>
     </row>

</xml_diff>